<commit_message>
docs(excel): matriz RACI de procesos de seguridad de la red
16 procesos (Gobernar a Recuperar) con R/A/C/I por rol de FinSegura, documento de
referencia y evidencia; una sola A por proceso. Hoja Roles con la asignación
propuesta al equipo según los commits (RSI y Admin IAM a definir). Bitácora del 07/10
actualizada.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/excel/04-bitacora-planilla.xlsx
+++ b/docs/excel/04-bitacora-planilla.xlsx
@@ -1008,7 +1008,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Bitácora (docs/99) y gestión de incidentes (docs/04, INC-2026-001..003); esta planilla y el registro de activos.</t>
+          <t>Bitácora (docs/99) y gestión de incidentes (docs/04, INC-2026-001..003); Excel de bitácora, registro de activos (A01-A22) y matriz RACI (16 procesos).</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
@@ -1018,7 +1018,7 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Borradores. Commit 0ba84e1; planillas en el commit siguiente</t>
+          <t>Borradores. Commits 0ba84e1, b3ba156 y siguiente</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">

</xml_diff>

<commit_message>
docs: Excel de controles MCU 5.0 e ISACA 01, 03, 07, 09
Excel 01: 47 controles del perfil Avanzado con Aplica, estado al 07/10 y evidencia o
brecha en el repo (5 implementados, 26 parciales, 15 pendientes, 1 N.A.), más hoja
Resumen por función con fórmulas (marcado para recalcular al abrir).

01 política, 03 riesgos (13 riesgos de brechas concretas del repo, 9 altos, con plan de
tratamiento), 07 monitoreo (1 de 8 fuentes de log verificada, retención sin configurar)
y 09 accesos (política de MFA/Argon2; opciones para el dashboard de Wazuh).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/excel/04-bitacora-planilla.xlsx
+++ b/docs/excel/04-bitacora-planilla.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Bitácora" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bitácora'!$A$1:$I$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bitácora'!$A$1:$I$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -18,8 +18,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -474,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1032,8 +1033,53 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="7" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Blue — Documentación</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>fmq203</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Excel 01 de controles MCU (47 controles + resumen) y documentos ISACA 01 política, 03 riesgos, 07 monitoreo, 09 accesos.</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>Borradores</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>Mismo día. Brechas nuevas: Suricata sin ruleset público, sin retención 90 d, imágenes :latest, egress sin restringir, MFA del dashboard de Wazuh sin camino definido.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I12"/>
+  <autoFilter ref="A1:I13"/>
   <dataValidations count="1">
     <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"S,N"</formula1>

</xml_diff>

<commit_message>
docs: notificación de incidentes (12) y estado actualizado
Criterios de decisión BCU/URCDP, evaluación registrada de INC-2026-001..003 (no
notificar: sin datos personales) y ejercicio de escritorio INC-2026-004 (exfiltración
de la base de clientes, CU-05) con los dos formularios completos. Plazos legales a
confirmar. INC-004 sumado al registro de 04; índice de docs, README, MEMORY y
bitácora (md y xlsx) al día.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/excel/04-bitacora-planilla.xlsx
+++ b/docs/excel/04-bitacora-planilla.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Bitácora" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bitácora'!$A$1:$I$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bitácora'!$A$1:$I$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1078,8 +1078,53 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="7" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Blue — Documentación</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>fmq203</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Kit de captura de evidencias (docs/evidencias/README.md); documentos 06 continuidad, 11 SoA (Anexo A completo, 93 controles), 12 notificación (ejercicio de escritorio INC-2026-004). Push al repo compartido.</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>git push</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Borradores</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>Mismo día. Evidencia no capturada (sin acceso de shell a docker-host desde la sesión). Sin respaldos de datos (RF-13). Plantilla SoA dice 79 controles; son 93.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I13"/>
+  <autoFilter ref="A1:I14"/>
   <dataValidations count="1">
     <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"S,N"</formula1>

</xml_diff>